<commit_message>
regjistri 17 i plotesuar
</commit_message>
<xml_diff>
--- a/Legalizim/4-Te-dhenat-per-kataster/regjistri/17-Regjistri-i-ndërrimeve-për-ndertesë-700-64-Verimi-Bibaj-Legalizim.xlsx
+++ b/Legalizim/4-Te-dhenat-per-kataster/regjistri/17-Regjistri-i-ndërrimeve-për-ndertesë-700-64-Verimi-Bibaj-Legalizim.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valon\OneDrive\Desktop\puna\Ferizaj\ferizaj\87-3-Verimi-Bibaj\700-64-Verimi-Bibja-Legalizim\4-Te-dhenat-per-kataster\regjistri\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valon\OneDrive\Desktop\puna\Ferizaj\ferizaj\87-3-Verimi-Bibaj\Legalizim\4-Te-dhenat-per-kataster\regjistri\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEA657C8-D7DF-4117-B5EC-D8548D184F51}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBA20A49-9501-4196-AD44-C9AC447F0A95}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="300" windowWidth="28440" windowHeight="15900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -105,9 +105,6 @@
     <t>Kati 1</t>
   </si>
   <si>
-    <t>ARAT E TJEGULLAVE</t>
-  </si>
-  <si>
     <t>Bibaj</t>
   </si>
   <si>
@@ -123,7 +120,10 @@
     <t>Rr. "Bau Bajden" -  Fsh. Bibaj - Ferizaj</t>
   </si>
   <si>
-    <t>VISAR (SHEFKI) AVDULLAHU</t>
+    <t>Ledinë</t>
+  </si>
+  <si>
+    <t>VISAR (KEMAJL) AVDULLAHU</t>
   </si>
 </sst>
 </file>
@@ -556,56 +556,8 @@
     <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -631,6 +583,39 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -640,8 +625,23 @@
     <xf numFmtId="2" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1087,170 +1087,170 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="20"/>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
+      <c r="A1" s="29"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" s="20"/>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-      <c r="O2" s="20"/>
-      <c r="P2" s="20"/>
+      <c r="A2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="29"/>
+      <c r="P2" s="29"/>
     </row>
     <row r="3" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="20"/>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
-      <c r="O3" s="20"/>
-      <c r="P3" s="20"/>
+      <c r="A3" s="29"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
-      <c r="O4" s="20"/>
-      <c r="P4" s="20"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="29"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="29"/>
+      <c r="P4" s="29"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A5" s="20"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
-      <c r="P5" s="20"/>
+      <c r="A5" s="29"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="29"/>
+      <c r="M5" s="29"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="29"/>
+      <c r="P5" s="29"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
-      <c r="N6" s="20"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
+      <c r="A6" s="29"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="29"/>
+      <c r="K6" s="29"/>
+      <c r="L6" s="29"/>
+      <c r="M6" s="29"/>
+      <c r="N6" s="29"/>
+      <c r="O6" s="29"/>
+      <c r="P6" s="29"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A7" s="20"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="20"/>
-      <c r="J7" s="20"/>
-      <c r="K7" s="20"/>
-      <c r="L7" s="20"/>
-      <c r="M7" s="20"/>
-      <c r="N7" s="20"/>
-      <c r="O7" s="20"/>
-      <c r="P7" s="20"/>
+      <c r="A7" s="29"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+      <c r="J7" s="29"/>
+      <c r="K7" s="29"/>
+      <c r="L7" s="29"/>
+      <c r="M7" s="29"/>
+      <c r="N7" s="29"/>
+      <c r="O7" s="29"/>
+      <c r="P7" s="29"/>
     </row>
     <row r="8" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="20"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="20"/>
-      <c r="L8" s="20"/>
-      <c r="M8" s="20"/>
-      <c r="N8" s="20"/>
-      <c r="O8" s="20"/>
-      <c r="P8" s="20"/>
+      <c r="A8" s="29"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="29"/>
+      <c r="K8" s="29"/>
+      <c r="L8" s="29"/>
+      <c r="M8" s="29"/>
+      <c r="N8" s="29"/>
+      <c r="O8" s="29"/>
+      <c r="P8" s="29"/>
     </row>
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
-      <c r="N9" s="22"/>
-      <c r="O9" s="22"/>
-      <c r="P9" s="23"/>
+      <c r="B9" s="31"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="31"/>
+      <c r="P9" s="32"/>
     </row>
     <row r="10" spans="1:17" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
@@ -1286,11 +1286,11 @@
       <c r="K10" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="L10" s="24" t="s">
+      <c r="L10" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="M10" s="24"/>
-      <c r="N10" s="24"/>
+      <c r="M10" s="33"/>
+      <c r="N10" s="33"/>
       <c r="O10" s="8" t="s">
         <v>9</v>
       </c>
@@ -1299,20 +1299,20 @@
       </c>
     </row>
     <row r="11" spans="1:17" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="28">
+      <c r="A11" s="37">
         <v>1</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="E11" s="34" t="s">
         <v>27</v>
-      </c>
-      <c r="E11" s="25" t="s">
-        <v>28</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>12</v>
@@ -1320,80 +1320,80 @@
       <c r="G11" s="14">
         <v>163.52600000000001</v>
       </c>
-      <c r="H11" s="45">
+      <c r="H11" s="40">
         <v>163.52600000000001</v>
       </c>
-      <c r="I11" s="25" t="s">
+      <c r="I11" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="J11" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="J11" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="K11" s="25" t="s">
+      <c r="K11" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="L11" s="34" t="s">
+      <c r="L11" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="M11" s="34"/>
-      <c r="N11" s="34"/>
-      <c r="O11" s="25">
+      <c r="M11" s="46"/>
+      <c r="N11" s="46"/>
+      <c r="O11" s="34">
         <v>1005029925</v>
       </c>
-      <c r="P11" s="31" t="s">
+      <c r="P11" s="43" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="29"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
+      <c r="A12" s="38"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
       <c r="F12" s="13" t="s">
         <v>24</v>
       </c>
       <c r="G12" s="11">
         <v>174.11</v>
       </c>
-      <c r="H12" s="46"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="35"/>
-      <c r="M12" s="35"/>
-      <c r="N12" s="35"/>
-      <c r="O12" s="26"/>
-      <c r="P12" s="32"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="35"/>
+      <c r="K12" s="35"/>
+      <c r="L12" s="47"/>
+      <c r="M12" s="47"/>
+      <c r="N12" s="47"/>
+      <c r="O12" s="35"/>
+      <c r="P12" s="44"/>
     </row>
     <row r="13" spans="1:17" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="29"/>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
+      <c r="A13" s="38"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
       <c r="F13" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G13" s="14">
         <v>136.85</v>
       </c>
-      <c r="H13" s="46"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="26"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="35"/>
-      <c r="M13" s="35"/>
-      <c r="N13" s="35"/>
-      <c r="O13" s="26"/>
-      <c r="P13" s="32"/>
+      <c r="H13" s="41"/>
+      <c r="I13" s="35"/>
+      <c r="J13" s="35"/>
+      <c r="K13" s="35"/>
+      <c r="L13" s="47"/>
+      <c r="M13" s="47"/>
+      <c r="N13" s="47"/>
+      <c r="O13" s="35"/>
+      <c r="P13" s="44"/>
     </row>
     <row r="14" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="30"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
+      <c r="A14" s="39"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
       <c r="F14" s="10" t="s">
         <v>20</v>
       </c>
@@ -1401,15 +1401,15 @@
         <f>SUM(G11:G13)</f>
         <v>474.48599999999999</v>
       </c>
-      <c r="H14" s="47"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
-      <c r="K14" s="27"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="27"/>
-      <c r="P14" s="33"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="36"/>
+      <c r="J14" s="36"/>
+      <c r="K14" s="36"/>
+      <c r="L14" s="48"/>
+      <c r="M14" s="48"/>
+      <c r="N14" s="48"/>
+      <c r="O14" s="36"/>
+      <c r="P14" s="45"/>
     </row>
     <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L15" s="1"/>
@@ -1427,74 +1427,74 @@
       <c r="Q16" s="15"/>
     </row>
     <row r="17" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="48"/>
+      <c r="D17" s="20"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
       <c r="P17" s="4"/>
       <c r="Q17" s="15"/>
     </row>
     <row r="18" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="48"/>
+      <c r="D18" s="20"/>
       <c r="F18" s="18"/>
       <c r="G18" s="19"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="15"/>
     </row>
     <row r="19" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D19" s="48"/>
+      <c r="D19" s="20"/>
       <c r="F19" s="18"/>
       <c r="G19" s="18"/>
       <c r="Q19" s="15"/>
     </row>
     <row r="20" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D20" s="48"/>
+      <c r="D20" s="20"/>
       <c r="Q20" s="16"/>
     </row>
     <row r="21" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="Q21" s="17"/>
     </row>
     <row r="22" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="41" t="s">
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="F22" s="41"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="41"/>
-      <c r="I22" s="41" t="s">
+      <c r="F22" s="25"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="25"/>
+      <c r="I22" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="J22" s="41"/>
-      <c r="K22" s="41"/>
-      <c r="L22" s="41"/>
-      <c r="M22" s="41"/>
-      <c r="N22" s="41"/>
-      <c r="O22" s="41"/>
-      <c r="P22" s="43"/>
+      <c r="J22" s="25"/>
+      <c r="K22" s="25"/>
+      <c r="L22" s="25"/>
+      <c r="M22" s="25"/>
+      <c r="N22" s="25"/>
+      <c r="O22" s="25"/>
+      <c r="P22" s="27"/>
       <c r="Q22" s="15"/>
     </row>
     <row r="23" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="39"/>
-      <c r="B23" s="40"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="42"/>
-      <c r="I23" s="42"/>
-      <c r="J23" s="42"/>
-      <c r="K23" s="42"/>
-      <c r="L23" s="42"/>
-      <c r="M23" s="42"/>
-      <c r="N23" s="42"/>
-      <c r="O23" s="42"/>
-      <c r="P23" s="44"/>
+      <c r="A23" s="23"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="26"/>
+      <c r="L23" s="26"/>
+      <c r="M23" s="26"/>
+      <c r="N23" s="26"/>
+      <c r="O23" s="26"/>
+      <c r="P23" s="28"/>
       <c r="Q23" s="15"/>
     </row>
     <row r="24" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1826,6 +1826,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="O11:O14"/>
+    <mergeCell ref="P11:P14"/>
+    <mergeCell ref="L11:N14"/>
     <mergeCell ref="A22:D23"/>
     <mergeCell ref="E22:H23"/>
     <mergeCell ref="I22:P23"/>
@@ -1842,9 +1845,6 @@
     <mergeCell ref="I11:I14"/>
     <mergeCell ref="J11:J14"/>
     <mergeCell ref="K11:K14"/>
-    <mergeCell ref="O11:O14"/>
-    <mergeCell ref="P11:P14"/>
-    <mergeCell ref="L11:N14"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>